<commit_message>
Added the experiment column
</commit_message>
<xml_diff>
--- a/docs/artificial data.xlsx
+++ b/docs/artificial data.xlsx
@@ -11,7 +11,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="90">
+  <si>
+    <t>Experiment</t>
+  </si>
   <si>
     <t>Date</t>
   </si>
@@ -38,6 +41,9 @@
   </si>
   <si>
     <t>Ground_Truth</t>
+  </si>
+  <si>
+    <t>Experiment_1</t>
   </si>
   <si>
     <t>17.08.2022</t>
@@ -166,6 +172,9 @@
 Tubular adenoma with low-grade dysplasia.
 Tubular adenoma with low-grade dysplasia, without evidence of malignancy in the examined specimen.
 Because the tissue was received in multiple fragments, the completeness of excision at the resection margins cannot be reliably assessed. Continued endoscopic surveillance is recommended according to the colonoscopy findings and established guidelines.</t>
+  </si>
+  <si>
+    <t>Experiment_2</t>
   </si>
   <si>
     <t>02.11.2019</t>
@@ -400,6 +409,9 @@
 Discharge Instructions:
 Oral antibiotic therapy according to the prescription, adequate hydration, rest, and follow-up with the primary care physician within 48–72 hours.
 The patient was advised to seek immediate medical evaluation in the event of worsening shortness of breath, significant chest pain, confusion, persistent fever, or reduced ability to maintain oral fluid intake.</t>
+  </si>
+  <si>
+    <t>Experiment_3</t>
   </si>
   <si>
     <t>12.06.2023</t>
@@ -1020,13 +1032,14 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="9.5"/>
-    <col customWidth="1" min="2" max="2" width="12.25"/>
-    <col customWidth="1" min="4" max="4" width="65.13"/>
-    <col customWidth="1" min="5" max="6" width="59.38"/>
-    <col customWidth="1" min="7" max="7" width="8.63"/>
-    <col customWidth="1" min="8" max="8" width="34.88"/>
-    <col customWidth="1" min="9" max="9" width="49.5"/>
+    <col customWidth="1" min="1" max="1" width="16.38"/>
+    <col customWidth="1" min="2" max="2" width="9.5"/>
+    <col customWidth="1" min="3" max="3" width="12.25"/>
+    <col customWidth="1" min="5" max="5" width="65.13"/>
+    <col customWidth="1" min="6" max="7" width="59.38"/>
+    <col customWidth="1" min="8" max="8" width="8.63"/>
+    <col customWidth="1" min="9" max="9" width="34.88"/>
+    <col customWidth="1" min="10" max="10" width="49.5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1057,291 +1070,324 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="4">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="4">
         <v>0.0</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="6" t="s">
-        <v>15</v>
+      <c r="I2" s="5"/>
+      <c r="J2" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="E3" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="F3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="4">
+        <v>22</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="4">
         <v>0.0</v>
       </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="6" t="s">
-        <v>22</v>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>30</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>35</v>
       </c>
+      <c r="D5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="6" t="s">
         <v>38</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>45</v>
+      <c r="H6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>47</v>
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="6" t="s">
         <v>53</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>55</v>
+        <v>33</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>62</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>79</v>
+        <v>65</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="12">
@@ -1349,18 +1395,21 @@
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
     </row>
     <row r="14">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>